<commit_message>
Google sheet app script integrated with Lead generate
</commit_message>
<xml_diff>
--- a/backend/leads.xlsx
+++ b/backend/leads.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -477,9 +477,35 @@
         <v>9/3/2026, 4:55:39 pm</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Testing</v>
+      </c>
+      <c r="B4" t="str">
+        <v>inhouse_ai@yopmail.com</v>
+      </c>
+      <c r="C4" t="str">
+        <v>91 8056746202</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>IT Services</v>
+      </c>
+      <c r="F4" t="str">
+        <v>India</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>10/3/2026, 10:05:52 am</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>